<commit_message>
flibe 0% li6 thf4 [250, 1000]
</commit_message>
<xml_diff>
--- a/Jupyter/Wedge/wedge_data_2026-03-02.xlsx
+++ b/Jupyter/Wedge/wedge_data_2026-03-02.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81856BF6-957C-4DAD-B08E-B588F3790719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-36" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="3" r:id="rId1"/>

</xml_diff>